<commit_message>
chore: Refatoração do código (Services adicionado)
</commit_message>
<xml_diff>
--- a/api/desempenho/2025-07-03.xlsx
+++ b/api/desempenho/2025-07-03.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -672,6 +672,258 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>15:32:23</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>26454</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>81.67</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>15:36:30</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>26752</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>81.45999999999999</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>15:39:51</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>26915</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>81.81999999999999</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>15:39:54</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>26915</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>85.17</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>15:41:03</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>26915</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>85.42</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>15:41:06</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>26915</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>85.55</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15:41:14</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>26915</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>85.67</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>15:41:14</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>26915</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>85.67</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>15:41:20</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>26915</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>85.67</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: Refatoração do código (SessionsService)
</commit_message>
<xml_diff>
--- a/api/desempenho/2025-07-03.xlsx
+++ b/api/desempenho/2025-07-03.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -924,6 +924,118 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>15:45:13</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>27327</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>82.20999999999999</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users-Mentores (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>15:45:16</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>27327</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>85.7</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota Users</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>15:50:34</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>27736</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>85.65000000000001</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota all_sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>15:54:29</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>28005</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>85.09</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota scheduled_sessions (VIEW)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: Refatoração do código - AvailabilityService.py
</commit_message>
<xml_diff>
--- a/api/desempenho/2025-07-03.xlsx
+++ b/api/desempenho/2025-07-03.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1036,6 +1036,90 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>15:56:56</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>28275</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>85.66</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota scheduled_sessions (VIEW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>15:56:58</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>28275</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>85.78</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Usuário acessou a rota all_sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>16:03:59</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>28661</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>127.0.0.1</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>85.31</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Acesso na AvailabilitySlot (mentor_id=db564152-c6c2-4c38-86fd-df738e1ba65c)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>